<commit_message>
adding more external sources
</commit_message>
<xml_diff>
--- a/fuentes_datos.xlsx
+++ b/fuentes_datos.xlsx
@@ -12,14 +12,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fuentes actuales'!$A$1:$G$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fuentes externas'!$A$1:$G$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fuentes externas'!$A$1:$G$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="155">
   <si>
     <t>Fuente</t>
   </si>
@@ -415,6 +415,60 @@
   </si>
   <si>
     <t>https://www.inegi.org.mx/programas/enaproce/2018/</t>
+  </si>
+  <si>
+    <t>Microdatos de Censos Económicos (Laboratorio de Microdatos)</t>
+  </si>
+  <si>
+    <t>Economía de CADA establecimiento: ingresos, gastos, remuneraciones, activos fijos y personal exacto (censos 2014/2019/2024). No públicos: acceso gratuito para posgrado/investigadores vía solicitud a microdatos@inegi.org.mx (CV + aval del director de tesis), presencial o procesamiento remoto; solo salen resultados agregados revisados por confidencialidad. La CLEE nace de estos censos → comparte identificador con el panel DENUE. Iniciar trámite con anticipación (tarda).</t>
+  </si>
+  <si>
+    <t>Establecimiento (dentro del entorno INEGI)</t>
+  </si>
+  <si>
+    <t>Candidata de alto valor — requiere trámite; complemento, no bloqueante</t>
+  </si>
+  <si>
+    <t>https://www.inegi.org.mx/microdatos/</t>
+  </si>
+  <si>
+    <t>SIEM (Sistema de Información Empresarial Mexicano)</t>
+  </si>
+  <si>
+    <t>Secretaría de Economía</t>
+  </si>
+  <si>
+    <t>Directorio de empresas registradas vía cámaras empresariales: contacto y giro, SIN información financiera y con cobertura sesgada (solo afiliadas). No aporta sobre lo que ya da DENUE.</t>
+  </si>
+  <si>
+    <t>Empresa (registro)</t>
+  </si>
+  <si>
+    <t>Continua</t>
+  </si>
+  <si>
+    <t>Descartada — sin datos económicos, cobertura sesgada</t>
+  </si>
+  <si>
+    <t>https://siem.economia.gob.mx/</t>
+  </si>
+  <si>
+    <t>Estados financieros de emisoras (BMV / BIVA)</t>
+  </si>
+  <si>
+    <t>BMV / BIVA / CNBV</t>
+  </si>
+  <si>
+    <t>Estados financieros completos, pero solo de ~140 empresas listadas en bolsa — irrelevante para micronegocios; el segmento no se traslapa con el objeto de estudio.</t>
+  </si>
+  <si>
+    <t>Empresa (solo emisoras)</t>
+  </si>
+  <si>
+    <t>Descartada — segmento no comparable</t>
+  </si>
+  <si>
+    <t>https://www.bmv.com.mx/</t>
   </si>
   <si>
     <t>Proyecciones de población municipal</t>
@@ -924,7 +978,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="38.7109375" customWidth="1"/>
@@ -1378,16 +1432,16 @@
         <v>132</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>56</v>
+        <v>8</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>133</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>29</v>
+        <v>134</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>134</v>
+        <v>71</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>135</v>
@@ -1396,8 +1450,77 @@
         <v>136</v>
       </c>
     </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G20"/>
+  <autoFilter ref="A1:G23"/>
   <hyperlinks>
     <hyperlink ref="G2" r:id="rId1"/>
     <hyperlink ref="G3" r:id="rId2"/>
@@ -1418,6 +1541,9 @@
     <hyperlink ref="G18" r:id="rId17"/>
     <hyperlink ref="G19" r:id="rId18"/>
     <hyperlink ref="G20" r:id="rId19"/>
+    <hyperlink ref="G21" r:id="rId20"/>
+    <hyperlink ref="G22" r:id="rId21"/>
+    <hyperlink ref="G23" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>